<commit_message>
New task labels and basic stats
</commit_message>
<xml_diff>
--- a/TaskACL.xlsx
+++ b/TaskACL.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/539fdd6ea201d1de/Documentos/Maestria/2025S/Phonetics TeamLab/DrunkenLinguists/inebriation-voice-detector/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="187" documentId="8_{C6B76E59-0855-4A4B-B150-0B21FA512158}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0CD65B20-1E21-44E5-9864-418CF193EF7E}"/>
+  <xr:revisionPtr revIDLastSave="327" documentId="8_{C6B76E59-0855-4A4B-B150-0B21FA512158}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E0324A2E-94F7-4DC5-B071-98A925AF7EDD}"/>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="2685" windowWidth="17430" windowHeight="11235" activeTab="2" xr2:uid="{1D073F97-6D20-42C2-8651-55E5ED9DD87A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{1D073F97-6D20-42C2-8651-55E5ED9DD87A}"/>
   </bookViews>
   <sheets>
     <sheet name="Match task" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="Sober tasks" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Drunk tasks'!$A$1:$G$31</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Sober tasks'!$A$1:$F$61</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -448,42 +449,27 @@
     <t>Please read the address: Ernst-Fahlbusch-Strasse 79, Göttingen Weende</t>
   </si>
   <si>
-    <t>Address</t>
-  </si>
-  <si>
     <t>Tell a story about the picture - tat_13MF</t>
   </si>
   <si>
     <t>Please read the phone number: 0862359286</t>
   </si>
   <si>
-    <t>Picture</t>
-  </si>
-  <si>
     <t>Please read as quickly as possible: A mossy trunk grows next to the stream, its sturdy, proud branch stretches upstream, pointing east and west.</t>
   </si>
   <si>
-    <t>Tonguetwister</t>
-  </si>
-  <si>
     <t>Please read the address: Sportplatzweg 27, Marktgraitz</t>
   </si>
   <si>
     <t>Please read the credit card number: 1390 7516 0281 9357</t>
   </si>
   <si>
-    <t>Number</t>
-  </si>
-  <si>
     <t>Talk to the experimenter about the picture - tat_3GF</t>
   </si>
   <si>
     <t>Please read the license plate number: STA-PB 2759</t>
   </si>
   <si>
-    <t>License plate</t>
-  </si>
-  <si>
     <t>Please read: Baker, Muselmann, People, Masses, Murderer, Moor, Mother, Manumentenmacher</t>
   </si>
   <si>
@@ -514,9 +500,6 @@
     <t>Please read the control command: Temperature 23 °C</t>
   </si>
   <si>
-    <t>Temperature</t>
-  </si>
-  <si>
     <t>Please imagine you want to tune the radio station to FM3. Command the car to do so.</t>
   </si>
   <si>
@@ -529,15 +512,9 @@
     <t>Please imagine you want to turn your seat heating to level 2. Command the car to do so.</t>
   </si>
   <si>
-    <t>Give command</t>
-  </si>
-  <si>
     <t>Please spell: M A R K T G R A I T Z</t>
   </si>
   <si>
-    <t>Spelling</t>
-  </si>
-  <si>
     <t>Please read the control command: Avoid highways.</t>
   </si>
   <si>
@@ -556,15 +533,6 @@
     <t>Reading</t>
   </si>
   <si>
-    <t>Fast list of words</t>
-  </si>
-  <si>
-    <t>Narrate</t>
-  </si>
-  <si>
-    <t>Command</t>
-  </si>
-  <si>
     <t>031</t>
   </si>
   <si>
@@ -914,6 +882,39 @@
   </si>
   <si>
     <t>061</t>
+  </si>
+  <si>
+    <t>Read an address</t>
+  </si>
+  <si>
+    <t>Read a command</t>
+  </si>
+  <si>
+    <t>Read a number</t>
+  </si>
+  <si>
+    <t>Read a tongue twister</t>
+  </si>
+  <si>
+    <t>Rapid word list</t>
+  </si>
+  <si>
+    <t>Read a license plate</t>
+  </si>
+  <si>
+    <t>Spell a word</t>
+  </si>
+  <si>
+    <t>Read a temperature</t>
+  </si>
+  <si>
+    <t>Issue a command</t>
+  </si>
+  <si>
+    <t>Tell a story</t>
+  </si>
+  <si>
+    <t>Describe an image</t>
   </si>
 </sst>
 </file>
@@ -1745,13 +1746,15 @@
     <col min="2" max="2" width="143.42578125" style="3" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="130.7109375" style="3" customWidth="1"/>
     <col min="4" max="4" width="21.140625" style="3" customWidth="1"/>
-    <col min="5" max="5" width="16" style="3" customWidth="1"/>
-    <col min="6" max="16384" width="9.140625" style="3"/>
+    <col min="5" max="5" width="20" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.28515625" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="9.140625" style="3"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>228</v>
+        <v>217</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>124</v>
@@ -1763,13 +1766,13 @@
         <v>131</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>271</v>
+        <v>260</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>289</v>
+        <v>278</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -1783,10 +1786,10 @@
         <v>129</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>143</v>
+        <v>282</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>93</v>
@@ -1800,7 +1803,7 @@
         <v>94</v>
       </c>
       <c r="B3" t="s">
-        <v>273</v>
+        <v>262</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>130</v>
@@ -1808,14 +1811,14 @@
       <c r="D3" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="E3" s="3" t="s">
-        <v>172</v>
+      <c r="E3" t="s">
+        <v>289</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>177</v>
+        <v>166</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>177</v>
+        <v>166</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -1823,22 +1826,22 @@
         <v>95</v>
       </c>
       <c r="B4" t="s">
-        <v>272</v>
+        <v>261</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>133</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>171</v>
+        <v>284</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>175</v>
+        <v>164</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>175</v>
+        <v>164</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -1846,19 +1849,19 @@
         <v>96</v>
       </c>
       <c r="B5" t="s">
-        <v>268</v>
+        <v>257</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>134</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>135</v>
+        <v>280</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>290</v>
+        <v>279</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -1866,16 +1869,16 @@
         <v>97</v>
       </c>
       <c r="B6" t="s">
-        <v>274</v>
+        <v>263</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>132</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>138</v>
+        <v>290</v>
       </c>
       <c r="F6" s="1" t="s">
         <v>122</v>
@@ -1892,13 +1895,13 @@
         <v>83</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>143</v>
+        <v>282</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>118</v>
@@ -1912,16 +1915,16 @@
         <v>99</v>
       </c>
       <c r="B8" t="s">
-        <v>275</v>
+        <v>264</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>140</v>
+        <v>162</v>
+      </c>
+      <c r="E8" t="s">
+        <v>283</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>115</v>
@@ -1938,13 +1941,13 @@
         <v>84</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>135</v>
+        <v>280</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>100</v>
@@ -1961,13 +1964,13 @@
         <v>85</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>143</v>
+        <v>282</v>
       </c>
       <c r="F10" s="1" t="s">
         <v>121</v>
@@ -1981,16 +1984,16 @@
         <v>102</v>
       </c>
       <c r="B11" t="s">
-        <v>276</v>
+        <v>265</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="D11" s="3" t="s">
         <v>132</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>138</v>
+        <v>290</v>
       </c>
       <c r="F11" s="1" t="s">
         <v>102</v>
@@ -2007,19 +2010,19 @@
         <v>86</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>146</v>
+        <v>285</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -2030,13 +2033,13 @@
         <v>123</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>171</v>
+        <v>284</v>
       </c>
       <c r="F13" s="1" t="s">
         <v>104</v>
@@ -2053,13 +2056,13 @@
         <v>87</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>135</v>
+        <v>280</v>
       </c>
       <c r="F14" s="1" t="s">
         <v>105</v>
@@ -2073,16 +2076,16 @@
         <v>106</v>
       </c>
       <c r="B15" t="s">
-        <v>278</v>
+        <v>267</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="D15" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="E15" s="3" t="s">
-        <v>172</v>
+      <c r="E15" t="s">
+        <v>289</v>
       </c>
       <c r="F15" s="1" t="s">
         <v>106</v>
@@ -2099,13 +2102,13 @@
         <v>88</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>143</v>
+        <v>282</v>
       </c>
       <c r="F16" s="1" t="s">
         <v>107</v>
@@ -2119,22 +2122,22 @@
         <v>108</v>
       </c>
       <c r="B17" t="s">
-        <v>277</v>
+        <v>266</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>140</v>
+        <v>162</v>
+      </c>
+      <c r="E17" t="s">
+        <v>283</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>179</v>
+        <v>168</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>179</v>
+        <v>168</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
@@ -2142,16 +2145,16 @@
         <v>109</v>
       </c>
       <c r="B18" t="s">
-        <v>266</v>
+        <v>255</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>135</v>
+        <v>280</v>
       </c>
       <c r="F18" s="1" t="s">
         <v>116</v>
@@ -2165,22 +2168,22 @@
         <v>110</v>
       </c>
       <c r="B19" t="s">
-        <v>279</v>
+        <v>268</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="D19" s="3" t="s">
         <v>132</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>138</v>
+        <v>290</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>181</v>
+        <v>170</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>181</v>
+        <v>170</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
@@ -2188,16 +2191,16 @@
         <v>111</v>
       </c>
       <c r="B20" t="s">
-        <v>267</v>
+        <v>256</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>135</v>
+        <v>280</v>
       </c>
       <c r="F20" s="1" t="s">
         <v>111</v>
@@ -2211,16 +2214,16 @@
         <v>112</v>
       </c>
       <c r="B21" t="s">
-        <v>281</v>
+        <v>270</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="E21" s="3" t="s">
-        <v>140</v>
+        <v>162</v>
+      </c>
+      <c r="E21" t="s">
+        <v>283</v>
       </c>
       <c r="F21" s="1" t="s">
         <v>112</v>
@@ -2234,22 +2237,22 @@
         <v>113</v>
       </c>
       <c r="B22" t="s">
-        <v>280</v>
+        <v>269</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>157</v>
+        <v>287</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>184</v>
+        <v>173</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>184</v>
+        <v>173</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
@@ -2260,19 +2263,19 @@
         <v>126</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="D23" s="3" t="s">
         <v>132</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>162</v>
+        <v>288</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>185</v>
+        <v>174</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>185</v>
+        <v>174</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
@@ -2280,22 +2283,22 @@
         <v>115</v>
       </c>
       <c r="B24" t="s">
-        <v>283</v>
+        <v>272</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>173</v>
+        <v>281</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>202</v>
+        <v>191</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>202</v>
+        <v>191</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
@@ -2306,19 +2309,19 @@
         <v>89</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>173</v>
+        <v>281</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>194</v>
+        <v>183</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>194</v>
+        <v>183</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
@@ -2329,19 +2332,19 @@
         <v>127</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="D26" s="3" t="s">
         <v>132</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>162</v>
+        <v>288</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>189</v>
+        <v>178</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>189</v>
+        <v>178</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
@@ -2349,22 +2352,22 @@
         <v>118</v>
       </c>
       <c r="B27" t="s">
-        <v>284</v>
+        <v>273</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>168</v>
+        <v>160</v>
       </c>
       <c r="D27" s="3" t="s">
         <v>132</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>162</v>
+        <v>288</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>198</v>
+        <v>187</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>198</v>
+        <v>187</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
@@ -2375,19 +2378,19 @@
         <v>90</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
       <c r="D28" s="3" t="s">
         <v>132</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>162</v>
+        <v>288</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>191</v>
+        <v>180</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>191</v>
+        <v>180</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
@@ -2395,22 +2398,22 @@
         <v>120</v>
       </c>
       <c r="B29" t="s">
-        <v>282</v>
+        <v>271</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="D29" s="3" t="s">
         <v>132</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>162</v>
+        <v>288</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>192</v>
+        <v>181</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>192</v>
+        <v>181</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
@@ -2421,19 +2424,19 @@
         <v>91</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>173</v>
+        <v>281</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>193</v>
+        <v>182</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>193</v>
+        <v>182</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
@@ -2444,22 +2447,23 @@
         <v>128</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>164</v>
+        <v>286</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>203</v>
+        <v>192</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>203</v>
+        <v>192</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:G31" xr:uid="{555EE763-D806-4242-80E0-FD997576B016}"/>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2474,13 +2478,13 @@
     <col min="2" max="2" width="143.42578125" customWidth="1"/>
     <col min="3" max="3" width="148" customWidth="1"/>
     <col min="4" max="4" width="14" customWidth="1"/>
-    <col min="5" max="5" width="16" customWidth="1"/>
+    <col min="5" max="5" width="20" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>271</v>
+        <v>260</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>124</v>
@@ -2492,13 +2496,13 @@
         <v>131</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>228</v>
+        <v>217</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>289</v>
+        <v>278</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -2512,10 +2516,10 @@
         <v>129</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>143</v>
+        <v>282</v>
       </c>
       <c r="F2" t="s">
         <v>93</v>
@@ -2529,16 +2533,16 @@
         <v>94</v>
       </c>
       <c r="B3" t="s">
-        <v>204</v>
+        <v>193</v>
       </c>
       <c r="C3" t="s">
-        <v>229</v>
+        <v>218</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>132</v>
       </c>
       <c r="E3" t="s">
-        <v>172</v>
+        <v>289</v>
       </c>
       <c r="G3" t="s">
         <v>94</v>
@@ -2549,16 +2553,16 @@
         <v>95</v>
       </c>
       <c r="B4" t="s">
-        <v>286</v>
+        <v>275</v>
       </c>
       <c r="C4" t="s">
-        <v>230</v>
+        <v>219</v>
       </c>
       <c r="D4" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="E4" t="s">
-        <v>140</v>
+        <v>283</v>
       </c>
       <c r="G4" t="s">
         <v>95</v>
@@ -2569,16 +2573,16 @@
         <v>96</v>
       </c>
       <c r="B5" t="s">
-        <v>261</v>
+        <v>250</v>
       </c>
       <c r="C5" t="s">
-        <v>231</v>
+        <v>220</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>135</v>
+        <v>280</v>
       </c>
       <c r="G5" t="s">
         <v>96</v>
@@ -2589,16 +2593,16 @@
         <v>97</v>
       </c>
       <c r="B6" t="s">
-        <v>287</v>
+        <v>276</v>
       </c>
       <c r="C6" t="s">
-        <v>232</v>
+        <v>221</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>132</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>138</v>
+        <v>290</v>
       </c>
       <c r="G6" t="s">
         <v>97</v>
@@ -2609,16 +2613,16 @@
         <v>98</v>
       </c>
       <c r="B7" t="s">
-        <v>205</v>
+        <v>194</v>
       </c>
       <c r="C7" t="s">
-        <v>233</v>
+        <v>222</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>143</v>
+        <v>282</v>
       </c>
       <c r="G7" t="s">
         <v>98</v>
@@ -2629,16 +2633,16 @@
         <v>99</v>
       </c>
       <c r="B8" t="s">
-        <v>206</v>
+        <v>195</v>
       </c>
       <c r="C8" t="s">
-        <v>234</v>
+        <v>223</v>
       </c>
       <c r="D8" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="E8" t="s">
-        <v>140</v>
+        <v>283</v>
       </c>
       <c r="G8" t="s">
         <v>99</v>
@@ -2652,13 +2656,13 @@
         <v>84</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>135</v>
+        <v>280</v>
       </c>
       <c r="F9" t="s">
         <v>100</v>
@@ -2672,16 +2676,16 @@
         <v>101</v>
       </c>
       <c r="B10" t="s">
-        <v>207</v>
+        <v>196</v>
       </c>
       <c r="C10" t="s">
-        <v>235</v>
+        <v>224</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>143</v>
+        <v>282</v>
       </c>
       <c r="G10" t="s">
         <v>101</v>
@@ -2692,16 +2696,16 @@
         <v>102</v>
       </c>
       <c r="B11" t="s">
-        <v>276</v>
+        <v>265</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="D11" s="3" t="s">
         <v>132</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>138</v>
+        <v>290</v>
       </c>
       <c r="F11" t="s">
         <v>102</v>
@@ -2715,16 +2719,16 @@
         <v>103</v>
       </c>
       <c r="B12" t="s">
-        <v>208</v>
+        <v>197</v>
       </c>
       <c r="C12" t="s">
-        <v>236</v>
+        <v>225</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>146</v>
+        <v>285</v>
       </c>
       <c r="G12" t="s">
         <v>103</v>
@@ -2738,13 +2742,13 @@
         <v>123</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>171</v>
+        <v>284</v>
       </c>
       <c r="F13" s="3" t="s">
         <v>104</v>
@@ -2761,13 +2765,13 @@
         <v>87</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>135</v>
+        <v>280</v>
       </c>
       <c r="F14" s="3" t="s">
         <v>105</v>
@@ -2781,16 +2785,16 @@
         <v>106</v>
       </c>
       <c r="B15" t="s">
-        <v>278</v>
+        <v>267</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="D15" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="E15" s="3" t="s">
-        <v>172</v>
+      <c r="E15" t="s">
+        <v>289</v>
       </c>
       <c r="F15" s="3" t="s">
         <v>106</v>
@@ -2807,13 +2811,13 @@
         <v>88</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>143</v>
+        <v>282</v>
       </c>
       <c r="F16" s="3" t="s">
         <v>107</v>
@@ -2827,16 +2831,16 @@
         <v>108</v>
       </c>
       <c r="B17" t="s">
-        <v>209</v>
+        <v>198</v>
       </c>
       <c r="C17" t="s">
-        <v>237</v>
+        <v>226</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="E17" t="s">
-        <v>140</v>
+        <v>283</v>
       </c>
       <c r="G17" t="s">
         <v>108</v>
@@ -2847,16 +2851,16 @@
         <v>109</v>
       </c>
       <c r="B18" t="s">
-        <v>269</v>
+        <v>258</v>
       </c>
       <c r="C18" t="s">
-        <v>238</v>
+        <v>227</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>135</v>
+        <v>280</v>
       </c>
       <c r="G18" t="s">
         <v>109</v>
@@ -2867,16 +2871,16 @@
         <v>110</v>
       </c>
       <c r="B19" t="s">
-        <v>288</v>
+        <v>277</v>
       </c>
       <c r="C19" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="D19" s="3" t="s">
         <v>132</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>138</v>
+        <v>290</v>
       </c>
       <c r="G19" t="s">
         <v>110</v>
@@ -2887,16 +2891,16 @@
         <v>111</v>
       </c>
       <c r="B20" t="s">
-        <v>262</v>
+        <v>251</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>135</v>
+        <v>280</v>
       </c>
       <c r="F20" s="3" t="s">
         <v>111</v>
@@ -2910,16 +2914,16 @@
         <v>112</v>
       </c>
       <c r="B21" t="s">
-        <v>281</v>
+        <v>270</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="E21" s="3" t="s">
-        <v>140</v>
+        <v>162</v>
+      </c>
+      <c r="E21" t="s">
+        <v>283</v>
       </c>
       <c r="F21" s="3" t="s">
         <v>112</v>
@@ -2933,16 +2937,16 @@
         <v>113</v>
       </c>
       <c r="B22" t="s">
-        <v>210</v>
+        <v>199</v>
       </c>
       <c r="C22" t="s">
-        <v>240</v>
+        <v>229</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>143</v>
+        <v>282</v>
       </c>
       <c r="G22" t="s">
         <v>113</v>
@@ -2953,16 +2957,16 @@
         <v>114</v>
       </c>
       <c r="B23" t="s">
-        <v>211</v>
+        <v>200</v>
       </c>
       <c r="C23" t="s">
-        <v>241</v>
+        <v>230</v>
       </c>
       <c r="D23" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="E23" s="3" t="s">
-        <v>172</v>
+      <c r="E23" t="s">
+        <v>289</v>
       </c>
       <c r="G23" t="s">
         <v>114</v>
@@ -2973,16 +2977,16 @@
         <v>115</v>
       </c>
       <c r="B24" t="s">
-        <v>275</v>
+        <v>264</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="E24" s="3" t="s">
-        <v>140</v>
+        <v>162</v>
+      </c>
+      <c r="E24" t="s">
+        <v>283</v>
       </c>
       <c r="F24" t="s">
         <v>99</v>
@@ -2996,16 +3000,16 @@
         <v>116</v>
       </c>
       <c r="B25" t="s">
-        <v>264</v>
+        <v>253</v>
       </c>
       <c r="C25" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>135</v>
+        <v>280</v>
       </c>
       <c r="F25" s="3" t="s">
         <v>109</v>
@@ -3019,16 +3023,16 @@
         <v>117</v>
       </c>
       <c r="B26" t="s">
-        <v>212</v>
+        <v>201</v>
       </c>
       <c r="C26" t="s">
-        <v>242</v>
+        <v>231</v>
       </c>
       <c r="D26" s="3" t="s">
         <v>132</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>138</v>
+        <v>290</v>
       </c>
       <c r="G26" t="s">
         <v>117</v>
@@ -3042,13 +3046,13 @@
         <v>83</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>143</v>
+        <v>282</v>
       </c>
       <c r="F27" s="3" t="s">
         <v>98</v>
@@ -3062,16 +3066,16 @@
         <v>119</v>
       </c>
       <c r="B28" t="s">
-        <v>213</v>
+        <v>202</v>
       </c>
       <c r="C28" t="s">
-        <v>243</v>
+        <v>232</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="E28" s="3" t="s">
-        <v>140</v>
+        <v>162</v>
+      </c>
+      <c r="E28" t="s">
+        <v>283</v>
       </c>
       <c r="G28" t="s">
         <v>119</v>
@@ -3082,16 +3086,16 @@
         <v>120</v>
       </c>
       <c r="B29" t="s">
-        <v>214</v>
+        <v>203</v>
       </c>
       <c r="C29" t="s">
-        <v>244</v>
+        <v>233</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>135</v>
+        <v>280</v>
       </c>
       <c r="G29" t="s">
         <v>120</v>
@@ -3105,13 +3109,13 @@
         <v>85</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>143</v>
+        <v>282</v>
       </c>
       <c r="F30" s="3" t="s">
         <v>101</v>
@@ -3125,16 +3129,16 @@
         <v>122</v>
       </c>
       <c r="B31" t="s">
-        <v>274</v>
+        <v>263</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D31" s="3" t="s">
         <v>132</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>138</v>
+        <v>290</v>
       </c>
       <c r="F31" s="3" t="s">
         <v>97</v>
@@ -3145,647 +3149,647 @@
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
       <c r="B32" t="s">
         <v>86</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>146</v>
+        <v>285</v>
       </c>
       <c r="F32" s="3" t="s">
         <v>103</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>175</v>
+        <v>164</v>
       </c>
       <c r="B33" t="s">
-        <v>272</v>
+        <v>261</v>
       </c>
       <c r="C33" s="3" t="s">
         <v>133</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>171</v>
+        <v>284</v>
       </c>
       <c r="F33" s="3" t="s">
         <v>95</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>175</v>
+        <v>164</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>176</v>
+        <v>165</v>
       </c>
       <c r="B34" t="s">
-        <v>265</v>
+        <v>254</v>
       </c>
       <c r="C34" t="s">
-        <v>245</v>
+        <v>234</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>135</v>
+        <v>280</v>
       </c>
       <c r="G34" t="s">
-        <v>176</v>
+        <v>165</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>177</v>
+        <v>166</v>
       </c>
       <c r="B35" t="s">
-        <v>285</v>
+        <v>274</v>
       </c>
       <c r="C35" t="s">
-        <v>246</v>
+        <v>235</v>
       </c>
       <c r="D35" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="E35" s="3" t="s">
-        <v>172</v>
+      <c r="E35" t="s">
+        <v>289</v>
       </c>
       <c r="F35" s="5" t="s">
         <v>94</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>177</v>
+        <v>166</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>178</v>
+        <v>167</v>
       </c>
       <c r="B36" t="s">
-        <v>215</v>
+        <v>204</v>
       </c>
       <c r="C36" t="s">
-        <v>247</v>
+        <v>236</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>143</v>
+        <v>282</v>
       </c>
       <c r="G36" t="s">
-        <v>178</v>
+        <v>167</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
-        <v>179</v>
+        <v>168</v>
       </c>
       <c r="B37" t="s">
-        <v>277</v>
+        <v>266</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="E37" s="3" t="s">
-        <v>140</v>
+        <v>162</v>
+      </c>
+      <c r="E37" t="s">
+        <v>283</v>
       </c>
       <c r="F37" s="3" t="s">
         <v>108</v>
       </c>
       <c r="G37" s="1" t="s">
-        <v>179</v>
+        <v>168</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>180</v>
+        <v>169</v>
       </c>
       <c r="B38" t="s">
-        <v>263</v>
+        <v>252</v>
       </c>
       <c r="C38" t="s">
-        <v>248</v>
+        <v>237</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>135</v>
+        <v>280</v>
       </c>
       <c r="G38" t="s">
-        <v>180</v>
+        <v>169</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>181</v>
+        <v>170</v>
       </c>
       <c r="B39" t="s">
-        <v>279</v>
+        <v>268</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="D39" s="3" t="s">
         <v>132</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>138</v>
+        <v>290</v>
       </c>
       <c r="F39" s="3" t="s">
         <v>110</v>
       </c>
       <c r="G39" s="1" t="s">
-        <v>181</v>
+        <v>170</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>182</v>
+        <v>171</v>
       </c>
       <c r="B40" t="s">
-        <v>270</v>
+        <v>259</v>
       </c>
       <c r="C40" t="s">
-        <v>249</v>
+        <v>238</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>135</v>
+        <v>280</v>
       </c>
       <c r="G40" t="s">
-        <v>182</v>
+        <v>171</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>183</v>
+        <v>172</v>
       </c>
       <c r="B41" t="s">
-        <v>216</v>
+        <v>205</v>
       </c>
       <c r="C41" t="s">
-        <v>250</v>
+        <v>239</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="E41" s="3" t="s">
-        <v>140</v>
+        <v>162</v>
+      </c>
+      <c r="E41" t="s">
+        <v>283</v>
       </c>
       <c r="G41" t="s">
-        <v>183</v>
+        <v>172</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
-        <v>184</v>
+        <v>173</v>
       </c>
       <c r="B42" t="s">
-        <v>280</v>
+        <v>269</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>157</v>
+        <v>287</v>
       </c>
       <c r="F42" s="3" t="s">
         <v>113</v>
       </c>
       <c r="G42" s="1" t="s">
-        <v>184</v>
+        <v>173</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
-        <v>185</v>
+        <v>174</v>
       </c>
       <c r="B43" t="s">
         <v>126</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="D43" s="3" t="s">
         <v>132</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>162</v>
+        <v>288</v>
       </c>
       <c r="F43" s="3" t="s">
         <v>114</v>
       </c>
       <c r="G43" s="1" t="s">
-        <v>185</v>
+        <v>174</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>186</v>
+        <v>175</v>
       </c>
       <c r="B44" t="s">
-        <v>217</v>
+        <v>206</v>
       </c>
       <c r="C44" t="s">
-        <v>251</v>
+        <v>240</v>
       </c>
       <c r="D44" s="3" t="s">
         <v>132</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>162</v>
+        <v>288</v>
       </c>
       <c r="G44" t="s">
-        <v>186</v>
+        <v>175</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>187</v>
+        <v>176</v>
       </c>
       <c r="B45" t="s">
-        <v>218</v>
+        <v>207</v>
       </c>
       <c r="C45" t="s">
-        <v>252</v>
+        <v>241</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>173</v>
+        <v>281</v>
       </c>
       <c r="G45" t="s">
-        <v>187</v>
+        <v>176</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>188</v>
+        <v>177</v>
       </c>
       <c r="B46" t="s">
-        <v>219</v>
+        <v>208</v>
       </c>
       <c r="C46" t="s">
-        <v>253</v>
+        <v>242</v>
       </c>
       <c r="D46" s="3" t="s">
         <v>132</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>162</v>
+        <v>288</v>
       </c>
       <c r="G46" t="s">
-        <v>188</v>
+        <v>177</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
-        <v>189</v>
+        <v>178</v>
       </c>
       <c r="B47" t="s">
         <v>127</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="D47" s="3" t="s">
         <v>132</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>162</v>
+        <v>288</v>
       </c>
       <c r="F47" s="3" t="s">
         <v>117</v>
       </c>
       <c r="G47" s="1" t="s">
-        <v>189</v>
+        <v>178</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>190</v>
+        <v>179</v>
       </c>
       <c r="B48" t="s">
-        <v>220</v>
+        <v>209</v>
       </c>
       <c r="C48" t="s">
-        <v>254</v>
+        <v>243</v>
       </c>
       <c r="D48" s="3" t="s">
         <v>132</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>162</v>
+        <v>288</v>
       </c>
       <c r="G48" t="s">
-        <v>190</v>
+        <v>179</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
-        <v>191</v>
+        <v>180</v>
       </c>
       <c r="B49" t="s">
-        <v>221</v>
+        <v>210</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
       <c r="D49" s="3" t="s">
         <v>132</v>
       </c>
       <c r="E49" s="3" t="s">
-        <v>162</v>
+        <v>288</v>
       </c>
       <c r="F49" s="3" t="s">
         <v>119</v>
       </c>
       <c r="G49" s="2" t="s">
-        <v>191</v>
+        <v>180</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
-        <v>192</v>
+        <v>181</v>
       </c>
       <c r="B50" t="s">
-        <v>282</v>
+        <v>271</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="D50" s="3" t="s">
         <v>132</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>162</v>
+        <v>288</v>
       </c>
       <c r="F50" s="3" t="s">
         <v>120</v>
       </c>
       <c r="G50" s="1" t="s">
-        <v>192</v>
+        <v>181</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
-        <v>193</v>
+        <v>182</v>
       </c>
       <c r="B51" t="s">
         <v>91</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>173</v>
+        <v>281</v>
       </c>
       <c r="F51" s="3" t="s">
         <v>121</v>
       </c>
       <c r="G51" s="1" t="s">
-        <v>193</v>
+        <v>182</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
-        <v>194</v>
+        <v>183</v>
       </c>
       <c r="B52" t="s">
         <v>89</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>173</v>
+        <v>281</v>
       </c>
       <c r="F52" s="3" t="s">
         <v>116</v>
       </c>
       <c r="G52" s="1" t="s">
-        <v>194</v>
+        <v>183</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>195</v>
+        <v>184</v>
       </c>
       <c r="B53" t="s">
-        <v>222</v>
+        <v>211</v>
       </c>
       <c r="C53" t="s">
-        <v>256</v>
+        <v>245</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>173</v>
+        <v>281</v>
       </c>
       <c r="G53" t="s">
-        <v>195</v>
+        <v>184</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>196</v>
+        <v>185</v>
       </c>
       <c r="B54" t="s">
-        <v>223</v>
+        <v>212</v>
       </c>
       <c r="C54" t="s">
-        <v>255</v>
+        <v>244</v>
       </c>
       <c r="D54" s="3" t="s">
         <v>132</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>162</v>
+        <v>288</v>
       </c>
       <c r="G54" t="s">
-        <v>196</v>
+        <v>185</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>197</v>
+        <v>186</v>
       </c>
       <c r="B55" t="s">
-        <v>224</v>
+        <v>213</v>
       </c>
       <c r="C55" t="s">
-        <v>257</v>
+        <v>246</v>
       </c>
       <c r="D55" s="3" t="s">
         <v>132</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>162</v>
+        <v>288</v>
       </c>
       <c r="G55" t="s">
-        <v>197</v>
+        <v>186</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
-        <v>198</v>
+        <v>187</v>
       </c>
       <c r="B56" t="s">
-        <v>284</v>
+        <v>273</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>168</v>
+        <v>160</v>
       </c>
       <c r="D56" s="3" t="s">
         <v>132</v>
       </c>
       <c r="E56" s="3" t="s">
-        <v>162</v>
+        <v>288</v>
       </c>
       <c r="F56" s="3" t="s">
         <v>118</v>
       </c>
       <c r="G56" s="1" t="s">
-        <v>198</v>
+        <v>187</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>199</v>
+        <v>188</v>
       </c>
       <c r="B57" t="s">
-        <v>225</v>
+        <v>214</v>
       </c>
       <c r="C57" t="s">
-        <v>258</v>
+        <v>247</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="E57" s="3" t="s">
-        <v>173</v>
+        <v>281</v>
       </c>
       <c r="G57" t="s">
-        <v>199</v>
+        <v>188</v>
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>200</v>
+        <v>189</v>
       </c>
       <c r="B58" t="s">
-        <v>226</v>
+        <v>215</v>
       </c>
       <c r="C58" t="s">
-        <v>259</v>
+        <v>248</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="E58" s="3" t="s">
-        <v>173</v>
+        <v>281</v>
       </c>
       <c r="G58" t="s">
-        <v>200</v>
+        <v>189</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>201</v>
+        <v>190</v>
       </c>
       <c r="B59" t="s">
-        <v>227</v>
+        <v>216</v>
       </c>
       <c r="C59" t="s">
-        <v>260</v>
+        <v>249</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="E59" s="3" t="s">
-        <v>173</v>
+        <v>281</v>
       </c>
       <c r="G59" t="s">
-        <v>201</v>
+        <v>190</v>
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
-        <v>202</v>
+        <v>191</v>
       </c>
       <c r="B60" t="s">
-        <v>283</v>
+        <v>272</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="E60" s="3" t="s">
-        <v>173</v>
+        <v>281</v>
       </c>
       <c r="F60" s="3" t="s">
         <v>115</v>
       </c>
       <c r="G60" s="1" t="s">
-        <v>202</v>
+        <v>191</v>
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
-        <v>203</v>
+        <v>192</v>
       </c>
       <c r="B61" t="s">
         <v>92</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="E61" s="3" t="s">
-        <v>164</v>
+        <v>286</v>
       </c>
       <c r="F61" s="3" t="s">
         <v>122</v>
       </c>
       <c r="G61" s="1" t="s">
-        <v>203</v>
+        <v>192</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Checking error rate to perform augmentation
</commit_message>
<xml_diff>
--- a/TaskACL.xlsx
+++ b/TaskACL.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/539fdd6ea201d1de/Documentos/Maestria/2025S/Phonetics TeamLab/DrunkenLinguists/inebriation-voice-detector/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="327" documentId="8_{C6B76E59-0855-4A4B-B150-0B21FA512158}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E0324A2E-94F7-4DC5-B071-98A925AF7EDD}"/>
+  <xr:revisionPtr revIDLastSave="331" documentId="8_{C6B76E59-0855-4A4B-B150-0B21FA512158}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DEFD38F3-ED71-43D9-B688-EACD1D452E52}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{1D073F97-6D20-42C2-8651-55E5ED9DD87A}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="10845" windowHeight="15585" firstSheet="1" activeTab="2" xr2:uid="{1D073F97-6D20-42C2-8651-55E5ED9DD87A}"/>
   </bookViews>
   <sheets>
     <sheet name="Match task" sheetId="1" r:id="rId1"/>
@@ -1743,10 +1743,10 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.42578125" style="3" customWidth="1"/>
-    <col min="2" max="2" width="143.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="143.42578125" style="3" customWidth="1"/>
     <col min="3" max="3" width="130.7109375" style="3" customWidth="1"/>
     <col min="4" max="4" width="21.140625" style="3" customWidth="1"/>
-    <col min="5" max="5" width="20" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20" style="3" customWidth="1"/>
     <col min="6" max="6" width="12.85546875" style="3" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="13.28515625" style="3" bestFit="1" customWidth="1"/>
     <col min="8" max="16384" width="9.140625" style="3"/>
@@ -2478,7 +2478,7 @@
     <col min="2" max="2" width="143.42578125" customWidth="1"/>
     <col min="3" max="3" width="148" customWidth="1"/>
     <col min="4" max="4" width="14" customWidth="1"/>
-    <col min="5" max="5" width="20" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20" customWidth="1"/>
     <col min="6" max="6" width="13.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>